<commit_message>
implementa orquestador canonico y valida pipeline operativo
</commit_message>
<xml_diff>
--- a/data/processed/modeling/encuestas_y_sentimiento_mensual_unificado.xlsx
+++ b/data/processed/modeling/encuestas_y_sentimiento_mensual_unificado.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mensual_unificado" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'mensual_unificado'!$A$1:$T$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'mensual_unificado'!$A$1:$T$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T19"/>
+  <dimension ref="A1:T20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1773,39 +1773,99 @@
       <c r="J19" s="3" t="inlineStr"/>
       <c r="K19" s="3" t="inlineStr"/>
       <c r="L19" t="n">
+        <v>4</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-W10</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-W13</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>0.7797959572845157</v>
+      </c>
+      <c r="P19" s="5" t="n">
+        <v>0.2004993413595564</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <v>-0.2193587134390587</v>
+      </c>
+      <c r="R19" s="5" t="n">
+        <v>0.1041126033256538</v>
+      </c>
+      <c r="S19" s="5" t="n">
+        <v>0.1240178669425632</v>
+      </c>
+      <c r="T19" s="5" t="n">
+        <v>0.1140652351341085</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ABRIL</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>46113</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" t="n">
         <v>1</v>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-W10</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>2026-W10</t>
-        </is>
-      </c>
-      <c r="O19" s="5" t="n">
-        <v>0.9565217391304348</v>
-      </c>
-      <c r="P19" s="5" t="n">
-        <v>0.08641975308641975</v>
-      </c>
-      <c r="Q19" s="5" t="n">
-        <v>-0.08942425479787669</v>
-      </c>
-      <c r="R19" s="5" t="n">
-        <v>0.2100585882774014</v>
-      </c>
-      <c r="S19" s="5" t="n">
-        <v>0.1278439869989166</v>
-      </c>
-      <c r="T19" s="5" t="n">
-        <v>0.168951287638159</v>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-W14</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-W14</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="n">
+        <v>0.7878787878787878</v>
+      </c>
+      <c r="P20" s="5" t="n">
+        <v>0.286624203821656</v>
+      </c>
+      <c r="Q20" s="5" t="n">
+        <v>-0.262483994878361</v>
+      </c>
+      <c r="R20" s="5" t="n">
+        <v>0.09355609798026393</v>
+      </c>
+      <c r="S20" s="5" t="n">
+        <v>0.1218498311249675</v>
+      </c>
+      <c r="T20" s="5" t="n">
+        <v>0.1077029645526157</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T19"/>
+  <autoFilter ref="A1:T20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>